<commit_message>
docs(demo-data): realistic dummy student names; a version for the demo college (Morning shift, as a new department), tested with the whole demo college: 397 classes, 0 clashes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo-data/GNDEC_CSE_3rd_4th_year_demo.xlsx
+++ b/docs/demo-data/GNDEC_CSE_3rd_4th_year_demo.xlsx
@@ -3734,7 +3734,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Student AA</t>
+          <t>Aarav Sharma</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Student AB</t>
+          <t>Aanya Dhillon</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Student AC</t>
+          <t>Arjun Mehta</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Student AD</t>
+          <t>Bhavya Kohli</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Student AE</t>
+          <t>Gurpreet Arora</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Student AF</t>
+          <t>Diya Bedi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Student AG</t>
+          <t>Harjot Saini</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Student AH</t>
+          <t>Gurleen Mann</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Student AI</t>
+          <t>Karan Grewal</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Student AJ</t>
+          <t>Harleen Kapoor</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Student AK</t>
+          <t>Manav Brar</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Student AL</t>
+          <t>Ishita Sandhu</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Student AM</t>
+          <t>Navdeep Malhotra</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Student AN</t>
+          <t>Jasleen Goyal</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Student AO</t>
+          <t>Rohan Thind</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Student AP</t>
+          <t>Kritika Bansal</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Student AQ</t>
+          <t>Sahil Sethi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4193,7 +4193,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Student AR</t>
+          <t>Mehak Walia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Student AS</t>
+          <t>Tejas Gill</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Student AT</t>
+          <t>Navneet Sidhu</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Student AU</t>
+          <t>Varun Jain</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Student AV</t>
+          <t>Prabhleen Ahuja</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Student AW</t>
+          <t>Yuvraj Verma</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Student AX</t>
+          <t>Riya Chopra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Student AY</t>
+          <t>Aman Bhatia</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Student AZ</t>
+          <t>Sanya Sharma</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Student AAA</t>
+          <t>Daksh Dhillon</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Student AAB</t>
+          <t>Tanvi Mehta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4490,7 +4490,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Student AAC</t>
+          <t>Ishaan Kohli</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Student AAD</t>
+          <t>Avneet Arora</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Student AAE</t>
+          <t>Jaskaran Bedi</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Student AAF</t>
+          <t>Simran Saini</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Student AAG</t>
+          <t>Kabir Mann</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Student AAH</t>
+          <t>Komal Grewal</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4652,7 +4652,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Student AAI</t>
+          <t>Lakshay Kapoor</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Student AAJ</t>
+          <t>Muskan Brar</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Student AAK</t>
+          <t>Parth Sandhu</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Student AAL</t>
+          <t>Nidhi Malhotra</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Student AAM</t>
+          <t>Ravneet Goyal</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Student AAN</t>
+          <t>Pooja Thind</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Student AAO</t>
+          <t>Simranjeet Bansal</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Student AAP</t>
+          <t>Ritika Sethi</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4868,7 +4868,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Student BA</t>
+          <t>Tanish Walia</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Student BB</t>
+          <t>Shreya Gill</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Student BC</t>
+          <t>Uday Sidhu</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Student BD</t>
+          <t>Tanya Jain</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Student BE</t>
+          <t>Vikram Ahuja</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Student BF</t>
+          <t>Vanshika Verma</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Student BG</t>
+          <t>Arshdeep Chopra</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Student BH</t>
+          <t>Anjali Bhatia</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Student BI</t>
+          <t>Bhavik Sharma</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Student BJ</t>
+          <t>Divya Dhillon</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Student BK</t>
+          <t>Dev Mehta</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Student BL</t>
+          <t>Ekam Kohli</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Student BM</t>
+          <t>Gagandeep Arora</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Student BN</t>
+          <t>Gunjan Bedi</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Student BO</t>
+          <t>Hardik Saini</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Student BP</t>
+          <t>Jasmeet Mann</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Student BQ</t>
+          <t>Inderjeet Grewal</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -5327,7 +5327,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Student BR</t>
+          <t>Manpreet Kapoor</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Student BS</t>
+          <t>Aarav Kohli</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Student BT</t>
+          <t>Aanya Arora</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Student BU</t>
+          <t>Arjun Bedi</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Student BV</t>
+          <t>Bhavya Saini</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Student BW</t>
+          <t>Gurpreet Mann</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Student BX</t>
+          <t>Diya Grewal</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Student BY</t>
+          <t>Harjot Kapoor</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Student BZ</t>
+          <t>Gurleen Brar</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Student BAA</t>
+          <t>Karan Sandhu</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -5597,7 +5597,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Student BAB</t>
+          <t>Harleen Malhotra</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Student BAC</t>
+          <t>Manav Goyal</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Student BAD</t>
+          <t>Ishita Thind</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Student BAE</t>
+          <t>Navdeep Bansal</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Student BAF</t>
+          <t>Jasleen Sethi</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Student BAG</t>
+          <t>Rohan Walia</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Student BAH</t>
+          <t>Kritika Gill</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Student BAI</t>
+          <t>Sahil Sidhu</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Student BAJ</t>
+          <t>Mehak Jain</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Student BAK</t>
+          <t>Tejas Ahuja</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Student BAL</t>
+          <t>Navneet Verma</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Student BAM</t>
+          <t>Varun Chopra</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Student BAN</t>
+          <t>Prabhleen Bhatia</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Student BAO</t>
+          <t>Yuvraj Sharma</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Student BAP</t>
+          <t>Riya Dhillon</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Student CA</t>
+          <t>Aman Mehta</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Student CB</t>
+          <t>Sanya Kohli</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Student CC</t>
+          <t>Daksh Arora</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Student CD</t>
+          <t>Tanvi Bedi</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Student CE</t>
+          <t>Ishaan Saini</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Student CF</t>
+          <t>Avneet Mann</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Student CG</t>
+          <t>Jaskaran Grewal</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Student CH</t>
+          <t>Simran Kapoor</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Student CI</t>
+          <t>Kabir Brar</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Student CJ</t>
+          <t>Komal Sandhu</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Student CK</t>
+          <t>Lakshay Malhotra</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -6299,7 +6299,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Student CL</t>
+          <t>Muskan Goyal</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Student CM</t>
+          <t>Parth Thind</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Student CN</t>
+          <t>Nidhi Bansal</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -6380,7 +6380,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Student CO</t>
+          <t>Ravneet Sethi</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Student CP</t>
+          <t>Pooja Walia</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -6434,7 +6434,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Student CQ</t>
+          <t>Simranjeet Gill</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Student CR</t>
+          <t>Ritika Sidhu</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -6488,7 +6488,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Student CS</t>
+          <t>Tanish Jain</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Student CT</t>
+          <t>Shreya Ahuja</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6542,7 +6542,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Student CU</t>
+          <t>Uday Verma</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -6569,7 +6569,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Student CV</t>
+          <t>Tanya Chopra</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6596,7 +6596,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Student CW</t>
+          <t>Vikram Bhatia</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Student CX</t>
+          <t>Vanshika Sharma</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Student CY</t>
+          <t>Arshdeep Dhillon</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Student CZ</t>
+          <t>Anjali Mehta</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Student CAA</t>
+          <t>Bhavik Kohli</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Student CAB</t>
+          <t>Divya Arora</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Student CAC</t>
+          <t>Dev Bedi</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Student CAD</t>
+          <t>Ekam Saini</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Student CAE</t>
+          <t>Gagandeep Mann</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Student CAF</t>
+          <t>Gunjan Grewal</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -6866,7 +6866,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Student CAG</t>
+          <t>Hardik Kapoor</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -6893,7 +6893,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Student CAH</t>
+          <t>Jasmeet Brar</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Student CAI</t>
+          <t>Inderjeet Sandhu</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Student CAJ</t>
+          <t>Manpreet Malhotra</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -6974,7 +6974,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Student CAK</t>
+          <t>Aarav Saini</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Student CAL</t>
+          <t>Aanya Mann</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Student CAM</t>
+          <t>Arjun Grewal</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Student CAN</t>
+          <t>Bhavya Kapoor</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Student CAO</t>
+          <t>Gurpreet Brar</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Student AA</t>
+          <t>Diya Sandhu</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Student AB</t>
+          <t>Harjot Malhotra</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Student AC</t>
+          <t>Gurleen Goyal</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Student AD</t>
+          <t>Karan Thind</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Student AE</t>
+          <t>Harleen Bansal</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Student AF</t>
+          <t>Manav Sethi</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Student AG</t>
+          <t>Ishita Walia</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Student AH</t>
+          <t>Navdeep Gill</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Student AI</t>
+          <t>Jasleen Sidhu</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Student AJ</t>
+          <t>Rohan Jain</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7379,7 +7379,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Student AK</t>
+          <t>Kritika Ahuja</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7406,7 +7406,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Student AL</t>
+          <t>Sahil Verma</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7433,7 +7433,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Student AM</t>
+          <t>Mehak Chopra</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Student AN</t>
+          <t>Tejas Bhatia</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Student AO</t>
+          <t>Navneet Sharma</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Student AP</t>
+          <t>Varun Dhillon</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7541,7 +7541,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Student AQ</t>
+          <t>Prabhleen Mehta</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Student AR</t>
+          <t>Yuvraj Kohli</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Student AS</t>
+          <t>Riya Arora</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Student AT</t>
+          <t>Aman Bedi</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -7649,7 +7649,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Student AU</t>
+          <t>Sanya Saini</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -7676,7 +7676,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Student AV</t>
+          <t>Daksh Mann</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -7703,7 +7703,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Student AW</t>
+          <t>Tanvi Grewal</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Student AX</t>
+          <t>Ishaan Kapoor</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Student AY</t>
+          <t>Avneet Brar</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -7784,7 +7784,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Student AZ</t>
+          <t>Jaskaran Sandhu</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Student AAA</t>
+          <t>Simran Malhotra</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Student AAB</t>
+          <t>Kabir Goyal</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Student AAC</t>
+          <t>Komal Thind</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Student AAD</t>
+          <t>Lakshay Bansal</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -7919,7 +7919,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Student AAE</t>
+          <t>Muskan Sethi</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -7946,7 +7946,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Student AAF</t>
+          <t>Parth Walia</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -7973,7 +7973,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Student AAG</t>
+          <t>Nidhi Gill</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -8000,7 +8000,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Student AAH</t>
+          <t>Ravneet Sidhu</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Student AAI</t>
+          <t>Pooja Jain</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Student AAJ</t>
+          <t>Simranjeet Ahuja</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -8081,7 +8081,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Student AAK</t>
+          <t>Ritika Verma</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Student AAL</t>
+          <t>Tanish Chopra</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Student AAM</t>
+          <t>Shreya Bhatia</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -8162,7 +8162,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Student AAN</t>
+          <t>Uday Sharma</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -8189,7 +8189,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Student AAO</t>
+          <t>Tanya Dhillon</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -8216,7 +8216,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Student AAP</t>
+          <t>Vikram Mehta</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Student BA</t>
+          <t>Vanshika Kohli</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Student BB</t>
+          <t>Arshdeep Arora</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -8297,7 +8297,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Student BC</t>
+          <t>Anjali Bedi</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -8324,7 +8324,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Student BD</t>
+          <t>Bhavik Saini</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Student BE</t>
+          <t>Divya Mann</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Student BF</t>
+          <t>Dev Grewal</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Student BG</t>
+          <t>Ekam Kapoor</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -8432,7 +8432,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Student BH</t>
+          <t>Gagandeep Brar</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -8459,7 +8459,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Student BI</t>
+          <t>Gunjan Sandhu</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -8486,7 +8486,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Student BJ</t>
+          <t>Hardik Malhotra</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Student BK</t>
+          <t>Jasmeet Goyal</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Student BL</t>
+          <t>Inderjeet Thind</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -8567,7 +8567,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Student BM</t>
+          <t>Manpreet Bansal</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -8594,7 +8594,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Student BN</t>
+          <t>Aarav Kapoor</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -8621,7 +8621,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Student BO</t>
+          <t>Aanya Brar</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Student BP</t>
+          <t>Arjun Sandhu</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Student BQ</t>
+          <t>Bhavya Malhotra</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Student BR</t>
+          <t>Gurpreet Goyal</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -8729,7 +8729,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Student BS</t>
+          <t>Diya Thind</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -8756,7 +8756,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Student BT</t>
+          <t>Harjot Bansal</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -8783,7 +8783,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Student BU</t>
+          <t>Gurleen Sethi</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Student BV</t>
+          <t>Karan Walia</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Student BW</t>
+          <t>Harleen Gill</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Student BX</t>
+          <t>Manav Sidhu</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -8891,7 +8891,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Student BY</t>
+          <t>Ishita Jain</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -8918,7 +8918,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Student BZ</t>
+          <t>Navdeep Ahuja</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Student BAA</t>
+          <t>Jasleen Verma</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -8972,7 +8972,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Student BAB</t>
+          <t>Rohan Chopra</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -8999,7 +8999,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Student BAC</t>
+          <t>Kritika Bhatia</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Student BAD</t>
+          <t>Sahil Sharma</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -9053,7 +9053,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Student BAE</t>
+          <t>Mehak Dhillon</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Student BAF</t>
+          <t>Tejas Mehta</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Student BAG</t>
+          <t>Navneet Kohli</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Student BAH</t>
+          <t>Varun Arora</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Student BAI</t>
+          <t>Prabhleen Bedi</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -9188,7 +9188,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Student BAJ</t>
+          <t>Yuvraj Saini</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Student BAK</t>
+          <t>Riya Mann</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -9242,7 +9242,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Student BAL</t>
+          <t>Aman Grewal</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -9269,7 +9269,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Student BAM</t>
+          <t>Sanya Kapoor</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Student BAN</t>
+          <t>Daksh Brar</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -9323,7 +9323,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Student BAO</t>
+          <t>Tanvi Sandhu</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Student BAP</t>
+          <t>Ishaan Malhotra</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -9377,7 +9377,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Student CA</t>
+          <t>Avneet Goyal</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -9404,7 +9404,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Student CB</t>
+          <t>Jaskaran Thind</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -9431,7 +9431,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Student CC</t>
+          <t>Simran Bansal</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Student CD</t>
+          <t>Kabir Sethi</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Student CE</t>
+          <t>Komal Walia</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -9512,7 +9512,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Student CF</t>
+          <t>Lakshay Gill</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Student CG</t>
+          <t>Muskan Sidhu</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Student CH</t>
+          <t>Parth Jain</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -9593,7 +9593,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Student CI</t>
+          <t>Nidhi Ahuja</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Student CJ</t>
+          <t>Ravneet Verma</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -9647,7 +9647,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Student CK</t>
+          <t>Pooja Chopra</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Student CL</t>
+          <t>Simranjeet Bhatia</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -9701,7 +9701,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Student CM</t>
+          <t>Ritika Sharma</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Student CN</t>
+          <t>Tanish Dhillon</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Student CO</t>
+          <t>Shreya Mehta</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -9782,7 +9782,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Student CP</t>
+          <t>Uday Kohli</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -9809,7 +9809,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Student CQ</t>
+          <t>Tanya Arora</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -9836,7 +9836,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Student CR</t>
+          <t>Vikram Bedi</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -9863,7 +9863,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Student CS</t>
+          <t>Vanshika Saini</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Student CT</t>
+          <t>Arshdeep Mann</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -9917,7 +9917,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Student CU</t>
+          <t>Anjali Grewal</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -9944,7 +9944,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Student CV</t>
+          <t>Bhavik Kapoor</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -9971,7 +9971,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Student CW</t>
+          <t>Divya Brar</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -9998,7 +9998,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Student CX</t>
+          <t>Dev Sandhu</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -10025,7 +10025,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Student CY</t>
+          <t>Ekam Malhotra</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -10052,7 +10052,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Student CZ</t>
+          <t>Gagandeep Goyal</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Student CAA</t>
+          <t>Gunjan Thind</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -10106,7 +10106,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Student CAB</t>
+          <t>Hardik Bansal</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Student CAC</t>
+          <t>Jasmeet Sethi</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -10160,7 +10160,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Student CAD</t>
+          <t>Inderjeet Walia</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Student CAE</t>
+          <t>Manpreet Gill</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Student CAF</t>
+          <t>Aarav Malhotra</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -10241,7 +10241,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Student CAG</t>
+          <t>Aanya Goyal</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -10268,7 +10268,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Student CAH</t>
+          <t>Arjun Thind</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Student CAI</t>
+          <t>Bhavya Bansal</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -10322,7 +10322,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Student CAJ</t>
+          <t>Gurpreet Sethi</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -10349,7 +10349,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Student CAK</t>
+          <t>Diya Walia</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -10376,7 +10376,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Student CAL</t>
+          <t>Harjot Gill</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -10403,7 +10403,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Student CAM</t>
+          <t>Gurleen Sidhu</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -10430,7 +10430,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Student CAN</t>
+          <t>Karan Jain</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -10457,7 +10457,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Student CAO</t>
+          <t>Harleen Ahuja</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">

</xml_diff>